<commit_message>
alteração planilha auth e codigos de apis para remover o campo session.
</commit_message>
<xml_diff>
--- a/auth.xlsx
+++ b/auth.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre.preis\Documents\Projeto_Bot_Vendas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAA9D189-9049-4C66-A0E5-4FE4F1BE32F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFB5DDCB-F62E-49C5-AFC5-2C2C196355A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,12 +20,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>number</t>
-  </si>
-  <si>
-    <t>session</t>
   </si>
   <si>
     <t>auth</t>
@@ -374,16 +371,15 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -393,9 +389,6 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>